<commit_message>
feat: Implement the Docs Agent feature, including document management, AI intent classification, Excel export, and associated UI components.
</commit_message>
<xml_diff>
--- a/nurotra workplace/Document_Feb22.xlsx
+++ b/nurotra workplace/Document_Feb22.xlsx
@@ -1,13 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_5AC27AE945D52FCF8ADB79CA566545B18651B11E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8848768F-49E8-4C13-BD94-CA5F673935FF}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Monthly Performance" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Strategic Analysis" state="visible" r:id="rId5"/>
+    <sheet name="Monthly Performance" sheetId="1" r:id="rId1"/>
+    <sheet name="Strategic Analysis" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -71,17 +86,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -445,11 +462,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -466,7 +483,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -477,15 +494,15 @@
         <v>32000</v>
       </c>
       <c r="D2">
-        <f>B2-C2</f>
+        <f t="shared" ref="D2:D7" si="0">B2-C2</f>
         <v>18000</v>
       </c>
-      <c r="E2" t="str">
-        <f>D2/B2</f>
-        <v>36%</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <f t="shared" ref="E2:E7" si="1">D2/B2</f>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -496,15 +513,15 @@
         <v>34000</v>
       </c>
       <c r="D3">
-        <f>B3-C3</f>
+        <f t="shared" si="0"/>
         <v>24000</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E3">
         <f>D3/B3</f>
-        <v>41%</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0.41379310344827586</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -515,15 +532,15 @@
         <v>31000</v>
       </c>
       <c r="D4">
-        <f>B4-C4</f>
+        <f t="shared" si="0"/>
         <v>14000</v>
       </c>
-      <c r="E4" t="str">
-        <f>D4/B4</f>
-        <v>31%</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>0.31111111111111112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -534,15 +551,15 @@
         <v>38000</v>
       </c>
       <c r="D5">
-        <f>B5-C5</f>
+        <f t="shared" si="0"/>
         <v>24000</v>
       </c>
-      <c r="E5" t="str">
-        <f>D5/B5</f>
-        <v>38%</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>0.38709677419354838</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -553,15 +570,15 @@
         <v>42000</v>
       </c>
       <c r="D6">
-        <f>B6-C6</f>
+        <f t="shared" si="0"/>
         <v>29000</v>
       </c>
-      <c r="E6" t="str">
-        <f>D6/B6</f>
-        <v>40%</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>0.40845070422535212</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -572,26 +589,26 @@
         <v>45000</v>
       </c>
       <c r="D7">
-        <f>B7-C7</f>
+        <f t="shared" si="0"/>
         <v>23000</v>
       </c>
-      <c r="E7" t="str">
-        <f>D7/B7</f>
-        <v>33%</v>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>0.33823529411764708</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -599,7 +616,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -608,7 +625,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -617,7 +634,7 @@
         <v>29000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -626,7 +643,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -635,17 +652,17 @@
         <v>354000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6" t="str">
         <f>IF(D6&gt;D2,"IMPROVING","DECLINING")</f>
-        <v>IMPROVING</v>
+        <v>DECLINING</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>